<commit_message>
feat(ai): restore and enhance Gemini AI assistant integration
</commit_message>
<xml_diff>
--- a/src/01-Operation/01_Operations_Standard/MASTER_DATABASE_UNIFICATO_2026.xlsx
+++ b/src/01-Operation/01_Operations_Standard/MASTER_DATABASE_UNIFICATO_2026.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30023"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30105"/>
   <workbookPr codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="4" documentId="11_71BBE02026CD82DDDA7484C4C4C871644B2242B4" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BA0F98A5-C792-4DAB-8808-7A7E4754837D}"/>
+  <xr:revisionPtr revIDLastSave="7" documentId="11_71BBE02026CD82DDDA7484C4C4C871644B2242B4" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7A821696-0796-4412-B10B-B11E8E9627FC}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" firstSheet="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Anagrafica Presidi" sheetId="1" r:id="rId1"/>
@@ -8474,7 +8474,7 @@
     <col min="10" max="10" width="26.625" customWidth="1"/>
     <col min="11" max="11" width="21.75" customWidth="1"/>
     <col min="12" max="12" width="18" customWidth="1"/>
-    <col min="13" max="13" width="177.625" customWidth="1"/>
+    <col min="13" max="13" width="74.125" customWidth="1"/>
     <col min="14" max="14" width="23.25" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>